<commit_message>
Excel export + charts: Sul de Minas by ENSO season
</commit_message>
<xml_diff>
--- a/exports/EspiritoSanto_ENSO_2006-2026.xlsx
+++ b/exports/EspiritoSanto_ENSO_2006-2026.xlsx
@@ -2465,11 +2465,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="24552787"/>
-        <c:axId val="56456277"/>
+        <c:axId val="51937505"/>
+        <c:axId val="43026028"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24552787"/>
+        <c:axId val="51937505"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2501,7 +2501,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56456277"/>
+        <c:crossAx val="43026028"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2509,7 +2509,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="56456277"/>
+        <c:axId val="43026028"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -2587,7 +2587,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24552787"/>
+        <c:crossAx val="51937505"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -4175,11 +4175,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="74520677"/>
-        <c:axId val="38876427"/>
+        <c:axId val="28888273"/>
+        <c:axId val="50334535"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="74520677"/>
+        <c:axId val="28888273"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4211,7 +4211,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38876427"/>
+        <c:crossAx val="50334535"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4219,7 +4219,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38876427"/>
+        <c:axId val="50334535"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="600"/>
@@ -4297,7 +4297,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74520677"/>
+        <c:crossAx val="28888273"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="100"/>
@@ -5915,11 +5915,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="39077572"/>
-        <c:axId val="34913693"/>
+        <c:axId val="80307702"/>
+        <c:axId val="83740633"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="39077572"/>
+        <c:axId val="80307702"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5951,7 +5951,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34913693"/>
+        <c:crossAx val="83740633"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5959,7 +5959,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34913693"/>
+        <c:axId val="83740633"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="600"/>
@@ -6037,7 +6037,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39077572"/>
+        <c:crossAx val="80307702"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="100"/>
@@ -7151,11 +7151,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="29994465"/>
-        <c:axId val="70140579"/>
+        <c:axId val="53646672"/>
+        <c:axId val="75321202"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="29994465"/>
+        <c:axId val="53646672"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7187,7 +7187,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70140579"/>
+        <c:crossAx val="75321202"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7195,7 +7195,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="70140579"/>
+        <c:axId val="75321202"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="600"/>
@@ -7273,7 +7273,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29994465"/>
+        <c:crossAx val="53646672"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="100"/>
@@ -8861,11 +8861,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="15431629"/>
-        <c:axId val="43478601"/>
+        <c:axId val="35152403"/>
+        <c:axId val="46769430"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="15431629"/>
+        <c:axId val="35152403"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8897,7 +8897,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43478601"/>
+        <c:crossAx val="46769430"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8905,7 +8905,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43478601"/>
+        <c:axId val="46769430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="90"/>
@@ -8983,7 +8983,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15431629"/>
+        <c:crossAx val="35152403"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -10601,11 +10601,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="16554373"/>
-        <c:axId val="34541370"/>
+        <c:axId val="80621190"/>
+        <c:axId val="32331731"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="16554373"/>
+        <c:axId val="80621190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10637,7 +10637,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34541370"/>
+        <c:crossAx val="32331731"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10645,7 +10645,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34541370"/>
+        <c:axId val="32331731"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="90"/>
@@ -10723,7 +10723,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16554373"/>
+        <c:crossAx val="80621190"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -11837,11 +11837,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="9005328"/>
-        <c:axId val="2444763"/>
+        <c:axId val="54434310"/>
+        <c:axId val="65700270"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="9005328"/>
+        <c:axId val="54434310"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11873,7 +11873,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2444763"/>
+        <c:crossAx val="65700270"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11881,7 +11881,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2444763"/>
+        <c:axId val="65700270"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="90"/>
@@ -11959,7 +11959,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9005328"/>
+        <c:crossAx val="54434310"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -13547,11 +13547,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="59279270"/>
-        <c:axId val="17158801"/>
+        <c:axId val="31059873"/>
+        <c:axId val="78094079"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="59279270"/>
+        <c:axId val="31059873"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13583,7 +13583,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17158801"/>
+        <c:crossAx val="78094079"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13591,7 +13591,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17158801"/>
+        <c:axId val="78094079"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="45"/>
@@ -13669,7 +13669,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59279270"/>
+        <c:crossAx val="31059873"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -15287,11 +15287,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47504944"/>
-        <c:axId val="76245238"/>
+        <c:axId val="12600789"/>
+        <c:axId val="24406438"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47504944"/>
+        <c:axId val="12600789"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15323,7 +15323,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76245238"/>
+        <c:crossAx val="24406438"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -15331,7 +15331,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76245238"/>
+        <c:axId val="24406438"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="45"/>
@@ -15409,7 +15409,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47504944"/>
+        <c:crossAx val="12600789"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -16523,11 +16523,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="89186925"/>
-        <c:axId val="84761509"/>
+        <c:axId val="14255031"/>
+        <c:axId val="6044871"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="89186925"/>
+        <c:axId val="14255031"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16559,7 +16559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84761509"/>
+        <c:crossAx val="6044871"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -16567,7 +16567,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84761509"/>
+        <c:axId val="6044871"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="45"/>
@@ -16645,7 +16645,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89186925"/>
+        <c:crossAx val="14255031"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -18263,11 +18263,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47152481"/>
-        <c:axId val="98263520"/>
+        <c:axId val="97175556"/>
+        <c:axId val="39316007"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47152481"/>
+        <c:axId val="97175556"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -18299,7 +18299,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98263520"/>
+        <c:crossAx val="39316007"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -18307,7 +18307,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98263520"/>
+        <c:axId val="39316007"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -18385,7 +18385,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47152481"/>
+        <c:crossAx val="97175556"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -19499,11 +19499,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="97450437"/>
-        <c:axId val="78415016"/>
+        <c:axId val="37633835"/>
+        <c:axId val="88340004"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="97450437"/>
+        <c:axId val="37633835"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -19535,7 +19535,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78415016"/>
+        <c:crossAx val="88340004"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -19543,7 +19543,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78415016"/>
+        <c:axId val="88340004"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -19621,7 +19621,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97450437"/>
+        <c:crossAx val="37633835"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -21209,11 +21209,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47413448"/>
-        <c:axId val="88512358"/>
+        <c:axId val="54555237"/>
+        <c:axId val="53108356"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47413448"/>
+        <c:axId val="54555237"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -21245,7 +21245,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88512358"/>
+        <c:crossAx val="53108356"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -21253,7 +21253,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88512358"/>
+        <c:axId val="53108356"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="26"/>
@@ -21331,7 +21331,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47413448"/>
+        <c:crossAx val="54555237"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -22949,11 +22949,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="93268876"/>
-        <c:axId val="7708704"/>
+        <c:axId val="91853340"/>
+        <c:axId val="77734100"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="93268876"/>
+        <c:axId val="91853340"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -22985,7 +22985,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7708704"/>
+        <c:crossAx val="77734100"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -22993,7 +22993,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7708704"/>
+        <c:axId val="77734100"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="26"/>
@@ -23071,7 +23071,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93268876"/>
+        <c:crossAx val="91853340"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -24185,11 +24185,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="91591196"/>
-        <c:axId val="15822191"/>
+        <c:axId val="47661782"/>
+        <c:axId val="65684747"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="91591196"/>
+        <c:axId val="47661782"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -24221,7 +24221,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15822191"/>
+        <c:crossAx val="65684747"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -24229,7 +24229,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15822191"/>
+        <c:axId val="65684747"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="26"/>
@@ -24307,7 +24307,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91591196"/>
+        <c:crossAx val="47661782"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -25895,11 +25895,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="33027460"/>
-        <c:axId val="19485278"/>
+        <c:axId val="40578182"/>
+        <c:axId val="21816121"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="33027460"/>
+        <c:axId val="40578182"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -25931,7 +25931,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19485278"/>
+        <c:crossAx val="21816121"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -25939,7 +25939,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19485278"/>
+        <c:axId val="21816121"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="36"/>
@@ -26017,7 +26017,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33027460"/>
+        <c:crossAx val="40578182"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -27635,11 +27635,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="55023020"/>
-        <c:axId val="87928415"/>
+        <c:axId val="31738696"/>
+        <c:axId val="36794058"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="55023020"/>
+        <c:axId val="31738696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -27671,7 +27671,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87928415"/>
+        <c:crossAx val="36794058"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -27679,7 +27679,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87928415"/>
+        <c:axId val="36794058"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="36"/>
@@ -27757,7 +27757,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55023020"/>
+        <c:crossAx val="31738696"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -28871,11 +28871,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="41394130"/>
-        <c:axId val="22837254"/>
+        <c:axId val="41393706"/>
+        <c:axId val="46463581"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="41394130"/>
+        <c:axId val="41393706"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -28907,7 +28907,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22837254"/>
+        <c:crossAx val="46463581"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -28915,7 +28915,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22837254"/>
+        <c:axId val="46463581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="36"/>
@@ -28993,7 +28993,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41394130"/>
+        <c:crossAx val="41393706"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>

</xml_diff>